<commit_message>
Rename 10mm HST to 200gr, fix Silvertip particle/suppression type
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changes/10mm-super.xlsx
+++ b/changes/10mm-super.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="113">
   <si>
     <t>10mm ammo scoring model</t>
   </si>
@@ -410,6 +410,9 @@
   </si>
   <si>
     <t>10mm Roosevelt Trailblazer 135gr Green Tracer</t>
+  </si>
+  <si>
+    <t>10mm_federal_hst_200gr_jhp</t>
   </si>
 </sst>
 </file>
@@ -2398,7 +2401,7 @@
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="54" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="B10" s="54" t="s">
         <v>101</v>

</xml_diff>